<commit_message>
adding wcgbts length and age target files
</commit_message>
<xml_diff>
--- a/2026/data/length_age_targets.xlsx
+++ b/2026/data/length_age_targets.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Claire.Rosemond\Documents\GitHub\survey_data_prioritization\2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2BF69AB-A5E6-4CB8-B417-02C91BE241C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6558B6C-42F9-4A90-987E-BD00F2731394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WCGBTS LENGTH TARGETS" sheetId="1" r:id="rId1"/>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1023,334 +1023,427 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W52"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
       <c r="B1">
-        <v>2003</v>
-      </c>
-      <c r="C1">
-        <v>2004</v>
-      </c>
-      <c r="D1">
-        <v>2005</v>
-      </c>
-      <c r="E1">
-        <v>2006</v>
-      </c>
-      <c r="F1">
-        <v>2007</v>
-      </c>
-      <c r="G1">
-        <v>2008</v>
-      </c>
-      <c r="H1">
-        <v>2009</v>
-      </c>
-      <c r="I1">
-        <v>2010</v>
-      </c>
-      <c r="J1">
-        <v>2011</v>
-      </c>
-      <c r="K1">
-        <v>2012</v>
-      </c>
-      <c r="L1">
-        <v>2013</v>
-      </c>
-      <c r="M1">
-        <v>2014</v>
-      </c>
-      <c r="N1">
-        <v>2015</v>
-      </c>
-      <c r="O1">
-        <v>2016</v>
-      </c>
-      <c r="P1">
-        <v>2017</v>
-      </c>
-      <c r="Q1">
-        <v>2018</v>
-      </c>
-      <c r="R1">
-        <v>2019</v>
-      </c>
-      <c r="S1">
-        <v>2021</v>
-      </c>
-      <c r="T1">
-        <v>2022</v>
-      </c>
-      <c r="U1">
-        <v>2023</v>
-      </c>
-      <c r="V1">
-        <v>2024</v>
-      </c>
-      <c r="W1">
         <v>2025</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B16">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B17">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B19">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B22">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B24">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B26">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B27">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B28">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B29">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B30">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B31">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B32">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B33">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B34">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B36">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B37">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B38">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B39">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B40">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B41">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B42">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B43">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B44">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B45">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B46">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B47">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B48">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B49">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B50">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B51">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>50</v>
+      </c>
+      <c r="B52">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1359,333 +1452,426 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W52"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
       <c r="B1">
-        <v>2003</v>
-      </c>
-      <c r="C1">
-        <v>2004</v>
-      </c>
-      <c r="D1">
-        <v>2005</v>
-      </c>
-      <c r="E1">
-        <v>2006</v>
-      </c>
-      <c r="F1">
-        <v>2007</v>
-      </c>
-      <c r="G1">
-        <v>2008</v>
-      </c>
-      <c r="H1">
-        <v>2009</v>
-      </c>
-      <c r="I1">
-        <v>2010</v>
-      </c>
-      <c r="J1">
-        <v>2011</v>
-      </c>
-      <c r="K1">
-        <v>2012</v>
-      </c>
-      <c r="L1">
-        <v>2013</v>
-      </c>
-      <c r="M1">
-        <v>2014</v>
-      </c>
-      <c r="N1">
-        <v>2015</v>
-      </c>
-      <c r="O1">
-        <v>2016</v>
-      </c>
-      <c r="P1">
-        <v>2017</v>
-      </c>
-      <c r="Q1">
-        <v>2018</v>
-      </c>
-      <c r="R1">
-        <v>2019</v>
-      </c>
-      <c r="S1">
-        <v>2021</v>
-      </c>
-      <c r="T1">
-        <v>2022</v>
-      </c>
-      <c r="U1">
-        <v>2023</v>
-      </c>
-      <c r="V1">
-        <v>2024</v>
-      </c>
-      <c r="W1">
         <v>2025</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B16">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B22">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B24">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B27">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B28">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B30">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B31">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B32">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B33">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B34">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B36">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B37">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B38">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B39">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B40">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B42">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B43">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B44">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B45">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B47">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B48">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B49">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B50">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B51">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>50</v>
+      </c>
+      <c r="B52">
         <v>50</v>
       </c>
     </row>
@@ -1695,152 +1881,89 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W52"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
       <c r="B1">
-        <v>2003</v>
-      </c>
-      <c r="C1">
-        <v>2004</v>
-      </c>
-      <c r="D1">
-        <v>2005</v>
-      </c>
-      <c r="E1">
-        <v>2006</v>
-      </c>
-      <c r="F1">
-        <v>2007</v>
-      </c>
-      <c r="G1">
-        <v>2008</v>
-      </c>
-      <c r="H1">
-        <v>2009</v>
-      </c>
-      <c r="I1">
-        <v>2010</v>
-      </c>
-      <c r="J1">
-        <v>2011</v>
-      </c>
-      <c r="K1">
-        <v>2012</v>
-      </c>
-      <c r="L1">
-        <v>2013</v>
-      </c>
-      <c r="M1">
-        <v>2014</v>
-      </c>
-      <c r="N1">
-        <v>2015</v>
-      </c>
-      <c r="O1">
-        <v>2016</v>
-      </c>
-      <c r="P1">
-        <v>2017</v>
-      </c>
-      <c r="Q1">
-        <v>2018</v>
-      </c>
-      <c r="R1">
-        <v>2019</v>
-      </c>
-      <c r="S1">
-        <v>2021</v>
-      </c>
-      <c r="T1">
-        <v>2022</v>
-      </c>
-      <c r="U1">
-        <v>2023</v>
-      </c>
-      <c r="V1">
-        <v>2024</v>
-      </c>
-      <c r="W1">
         <v>2025</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2031,152 +2154,89 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W52"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>51</v>
       </c>
       <c r="B1">
-        <v>2003</v>
-      </c>
-      <c r="C1">
-        <v>2004</v>
-      </c>
-      <c r="D1">
-        <v>2005</v>
-      </c>
-      <c r="E1">
-        <v>2006</v>
-      </c>
-      <c r="F1">
-        <v>2007</v>
-      </c>
-      <c r="G1">
-        <v>2008</v>
-      </c>
-      <c r="H1">
-        <v>2009</v>
-      </c>
-      <c r="I1">
-        <v>2010</v>
-      </c>
-      <c r="J1">
-        <v>2011</v>
-      </c>
-      <c r="K1">
-        <v>2012</v>
-      </c>
-      <c r="L1">
-        <v>2013</v>
-      </c>
-      <c r="M1">
-        <v>2014</v>
-      </c>
-      <c r="N1">
-        <v>2015</v>
-      </c>
-      <c r="O1">
-        <v>2016</v>
-      </c>
-      <c r="P1">
-        <v>2017</v>
-      </c>
-      <c r="Q1">
-        <v>2018</v>
-      </c>
-      <c r="R1">
-        <v>2019</v>
-      </c>
-      <c r="S1">
-        <v>2021</v>
-      </c>
-      <c r="T1">
-        <v>2022</v>
-      </c>
-      <c r="U1">
-        <v>2023</v>
-      </c>
-      <c r="V1">
-        <v>2024</v>
-      </c>
-      <c r="W1">
         <v>2025</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>

</xml_diff>